<commit_message>
Updated report and other handlings
</commit_message>
<xml_diff>
--- a/usn_list.xlsx
+++ b/usn_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\india\Desktop\VTU_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56D6E0E3-174E-414F-8337-E205AC662AFB}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{198F875D-B20D-431A-B771-C65E3F67AB2C}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3D3C98C4-02F0-4FB4-9D88-793BC642E170}"/>
   </bookViews>
@@ -30,18 +30,189 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t>USN</t>
   </si>
   <si>
-    <t>1XX22XX000</t>
-  </si>
-  <si>
     <t>1XX22XX001</t>
   </si>
   <si>
     <t>1XX22XX002</t>
+  </si>
+  <si>
+    <t>1XX22XX003</t>
+  </si>
+  <si>
+    <t>1XX22XX004</t>
+  </si>
+  <si>
+    <t>1XX22XX005</t>
+  </si>
+  <si>
+    <t>1XX22XX006</t>
+  </si>
+  <si>
+    <t>1XX22XX007</t>
+  </si>
+  <si>
+    <t>1XX22XX008</t>
+  </si>
+  <si>
+    <t>1XX22XX009</t>
+  </si>
+  <si>
+    <t>1XX22XX010</t>
+  </si>
+  <si>
+    <t>1XX22XX011</t>
+  </si>
+  <si>
+    <t>1XX22XX012</t>
+  </si>
+  <si>
+    <t>1XX22XX013</t>
+  </si>
+  <si>
+    <t>1XX22XX014</t>
+  </si>
+  <si>
+    <t>1XX22XX015</t>
+  </si>
+  <si>
+    <t>1XX22XX016</t>
+  </si>
+  <si>
+    <t>1XX22XX017</t>
+  </si>
+  <si>
+    <t>1XX22XX018</t>
+  </si>
+  <si>
+    <t>1XX22XX019</t>
+  </si>
+  <si>
+    <t>1XX22XX020</t>
+  </si>
+  <si>
+    <t>1XX22XX021</t>
+  </si>
+  <si>
+    <t>1XX22XX022</t>
+  </si>
+  <si>
+    <t>1XX22XX023</t>
+  </si>
+  <si>
+    <t>1XX22XX024</t>
+  </si>
+  <si>
+    <t>1XX22XX025</t>
+  </si>
+  <si>
+    <t>1XX22XX026</t>
+  </si>
+  <si>
+    <t>1XX22XX027</t>
+  </si>
+  <si>
+    <t>1XX22XX028</t>
+  </si>
+  <si>
+    <t>1XX22XX029</t>
+  </si>
+  <si>
+    <t>1XX22XX030</t>
+  </si>
+  <si>
+    <t>1XX22XX031</t>
+  </si>
+  <si>
+    <t>1XX22XX032</t>
+  </si>
+  <si>
+    <t>1XX22XX033</t>
+  </si>
+  <si>
+    <t>1XX22XX034</t>
+  </si>
+  <si>
+    <t>1XX22XX035</t>
+  </si>
+  <si>
+    <t>1XX22XX036</t>
+  </si>
+  <si>
+    <t>1XX22XX037</t>
+  </si>
+  <si>
+    <t>1XX22XX038</t>
+  </si>
+  <si>
+    <t>1XX22XX039</t>
+  </si>
+  <si>
+    <t>1XX22XX040</t>
+  </si>
+  <si>
+    <t>1XX22XX041</t>
+  </si>
+  <si>
+    <t>1XX22XX042</t>
+  </si>
+  <si>
+    <t>1XX22XX043</t>
+  </si>
+  <si>
+    <t>1XX22XX044</t>
+  </si>
+  <si>
+    <t>1XX22XX045</t>
+  </si>
+  <si>
+    <t>1XX22XX046</t>
+  </si>
+  <si>
+    <t>1XX22XX047</t>
+  </si>
+  <si>
+    <t>1XX22XX048</t>
+  </si>
+  <si>
+    <t>1XX22XX049</t>
+  </si>
+  <si>
+    <t>1XX22XX050</t>
+  </si>
+  <si>
+    <t>1XX22XX051</t>
+  </si>
+  <si>
+    <t>1XX22XX052</t>
+  </si>
+  <si>
+    <t>1XX22XX053</t>
+  </si>
+  <si>
+    <t>1XX22XX054</t>
+  </si>
+  <si>
+    <t>1XX22XX055</t>
+  </si>
+  <si>
+    <t>1XX22XX056</t>
+  </si>
+  <si>
+    <t>1XX22XX057</t>
+  </si>
+  <si>
+    <t>1XX22XX058</t>
+  </si>
+  <si>
+    <t>1XX22XX059</t>
+  </si>
+  <si>
+    <t>1XX22XX060</t>
   </si>
 </sst>
 </file>
@@ -399,7 +570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75035D5B-D679-4EC4-BC71-1582A31A3314}">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.140625" customWidth="1"/>
@@ -425,6 +596,291 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>